<commit_message>
📊 Actualizar CV_PF.xlsx — 25-03-2026, 10:00:20 a. m.
</commit_message>
<xml_diff>
--- a/datos/CV_PF.xlsx
+++ b/datos/CV_PF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF6F809D-2ED1-4770-811E-EBB475309F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5FEA576D-D88B-4BEE-B0BD-C8C25729F120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2226" uniqueCount="677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2478" uniqueCount="717">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -2051,6 +2051,126 @@
   </si>
   <si>
     <t>3964</t>
+  </si>
+  <si>
+    <t>4137131-5</t>
+  </si>
+  <si>
+    <t>ARANCIBIA GAMBOA ROBERTO JAIME</t>
+  </si>
+  <si>
+    <t>10/08/1942</t>
+  </si>
+  <si>
+    <t>Pedro Aguirre Cerda</t>
+  </si>
+  <si>
+    <t>6132 - Pedro Aguirre Cerda - Santiago -CP</t>
+  </si>
+  <si>
+    <t>936398005</t>
+  </si>
+  <si>
+    <t>rarancibia430@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>23/03/2026</t>
+  </si>
+  <si>
+    <t>Yohany Margarita Gonzalez Rojas</t>
+  </si>
+  <si>
+    <t>27458</t>
+  </si>
+  <si>
+    <t>3968</t>
+  </si>
+  <si>
+    <t>6155513-7</t>
+  </si>
+  <si>
+    <t>TAMBLEY ROMERO JORGE HERNAN</t>
+  </si>
+  <si>
+    <t>03/09/1952</t>
+  </si>
+  <si>
+    <t>890 - San Miguel - Santiago -CP</t>
+  </si>
+  <si>
+    <t>979572729</t>
+  </si>
+  <si>
+    <t>jhtambleyr@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>360000</t>
+  </si>
+  <si>
+    <t>3976</t>
+  </si>
+  <si>
+    <t>3977</t>
+  </si>
+  <si>
+    <t>257000</t>
+  </si>
+  <si>
+    <t>2308000</t>
+  </si>
+  <si>
+    <t>64111</t>
+  </si>
+  <si>
+    <t>3978</t>
+  </si>
+  <si>
+    <t>8561974-8</t>
+  </si>
+  <si>
+    <t>JIMENEZ GIULIUCCI LEONARDO DE JESUS</t>
+  </si>
+  <si>
+    <t>15/10/1960</t>
+  </si>
+  <si>
+    <t>9471 - La Florida - Santiago -CP</t>
+  </si>
+  <si>
+    <t>974468599</t>
+  </si>
+  <si>
+    <t>leo.jigi@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>1450000</t>
+  </si>
+  <si>
+    <t>1218487</t>
+  </si>
+  <si>
+    <t>3981</t>
+  </si>
+  <si>
+    <t>7545444-9</t>
+  </si>
+  <si>
+    <t>CONTRERAS GONZALEZ MARÍA ANGELICA</t>
+  </si>
+  <si>
+    <t>06/02/1957</t>
+  </si>
+  <si>
+    <t>989100567</t>
+  </si>
+  <si>
+    <t>macggo@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>24/03/2026</t>
+  </si>
+  <si>
+    <t>3994</t>
   </si>
 </sst>
 </file>
@@ -2911,11 +3031,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP53"/>
+  <dimension ref="A1:AP59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="41" width="8" customWidth="1"/>
-    <col min="42" max="42" width="12" customWidth="1"/>
+    <col min="1" max="42" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.3">
@@ -9276,7 +9395,7 @@
         <v>638</v>
       </c>
       <c r="AC50" t="s">
-        <v>103</v>
+        <v>62</v>
       </c>
       <c r="AD50" t="s">
         <v>261</v>
@@ -9404,7 +9523,7 @@
         <v>648</v>
       </c>
       <c r="AC51" t="s">
-        <v>103</v>
+        <v>62</v>
       </c>
       <c r="AD51" t="s">
         <v>651</v>
@@ -9700,6 +9819,774 @@
       </c>
       <c r="AP53" t="s">
         <v>676</v>
+      </c>
+    </row>
+    <row r="54" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>42</v>
+      </c>
+      <c r="B54" t="s">
+        <v>43</v>
+      </c>
+      <c r="C54" t="s">
+        <v>677</v>
+      </c>
+      <c r="D54" t="s">
+        <v>678</v>
+      </c>
+      <c r="E54" t="s">
+        <v>679</v>
+      </c>
+      <c r="F54" t="s">
+        <v>680</v>
+      </c>
+      <c r="G54" t="s">
+        <v>681</v>
+      </c>
+      <c r="H54" t="s">
+        <v>49</v>
+      </c>
+      <c r="I54" t="s">
+        <v>682</v>
+      </c>
+      <c r="J54" t="s">
+        <v>683</v>
+      </c>
+      <c r="K54" t="s">
+        <v>659</v>
+      </c>
+      <c r="L54" t="s">
+        <v>684</v>
+      </c>
+      <c r="M54" t="s">
+        <v>53</v>
+      </c>
+      <c r="N54" t="s">
+        <v>54</v>
+      </c>
+      <c r="O54" t="s">
+        <v>397</v>
+      </c>
+      <c r="P54" t="s">
+        <v>685</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>626</v>
+      </c>
+      <c r="R54" t="s">
+        <v>482</v>
+      </c>
+      <c r="S54" t="s">
+        <v>49</v>
+      </c>
+      <c r="T54" t="s">
+        <v>511</v>
+      </c>
+      <c r="U54" t="s">
+        <v>57</v>
+      </c>
+      <c r="V54" t="s">
+        <v>57</v>
+      </c>
+      <c r="W54" t="s">
+        <v>164</v>
+      </c>
+      <c r="X54" t="s">
+        <v>538</v>
+      </c>
+      <c r="Y54" t="s">
+        <v>684</v>
+      </c>
+      <c r="Z54" t="s">
+        <v>349</v>
+      </c>
+      <c r="AA54" t="s">
+        <v>179</v>
+      </c>
+      <c r="AB54" t="s">
+        <v>686</v>
+      </c>
+      <c r="AC54" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD54" t="s">
+        <v>104</v>
+      </c>
+      <c r="AE54" t="s">
+        <v>84</v>
+      </c>
+      <c r="AF54" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG54" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH54" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI54" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ54" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK54" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL54" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM54" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN54" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO54" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP54" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="55" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>42</v>
+      </c>
+      <c r="B55" t="s">
+        <v>43</v>
+      </c>
+      <c r="C55" t="s">
+        <v>688</v>
+      </c>
+      <c r="D55" t="s">
+        <v>689</v>
+      </c>
+      <c r="E55" t="s">
+        <v>690</v>
+      </c>
+      <c r="F55" t="s">
+        <v>633</v>
+      </c>
+      <c r="G55" t="s">
+        <v>691</v>
+      </c>
+      <c r="H55" t="s">
+        <v>692</v>
+      </c>
+      <c r="I55" t="s">
+        <v>692</v>
+      </c>
+      <c r="J55" t="s">
+        <v>693</v>
+      </c>
+      <c r="K55" t="s">
+        <v>684</v>
+      </c>
+      <c r="L55" t="s">
+        <v>684</v>
+      </c>
+      <c r="M55" t="s">
+        <v>53</v>
+      </c>
+      <c r="N55" t="s">
+        <v>54</v>
+      </c>
+      <c r="O55" t="s">
+        <v>55</v>
+      </c>
+      <c r="P55" t="s">
+        <v>318</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>179</v>
+      </c>
+      <c r="R55" t="s">
+        <v>479</v>
+      </c>
+      <c r="S55" t="s">
+        <v>49</v>
+      </c>
+      <c r="T55" t="s">
+        <v>480</v>
+      </c>
+      <c r="U55" t="s">
+        <v>57</v>
+      </c>
+      <c r="V55" t="s">
+        <v>57</v>
+      </c>
+      <c r="W55" t="s">
+        <v>164</v>
+      </c>
+      <c r="X55" t="s">
+        <v>481</v>
+      </c>
+      <c r="Y55" t="s">
+        <v>684</v>
+      </c>
+      <c r="Z55" t="s">
+        <v>482</v>
+      </c>
+      <c r="AA55" t="s">
+        <v>179</v>
+      </c>
+      <c r="AB55" t="s">
+        <v>694</v>
+      </c>
+      <c r="AC55" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD55" t="s">
+        <v>104</v>
+      </c>
+      <c r="AE55" t="s">
+        <v>84</v>
+      </c>
+      <c r="AF55" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG55" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH55" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI55" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ55" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK55" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL55" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM55" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN55" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO55" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP55" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="56" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>42</v>
+      </c>
+      <c r="B56" t="s">
+        <v>43</v>
+      </c>
+      <c r="C56" t="s">
+        <v>688</v>
+      </c>
+      <c r="D56" t="s">
+        <v>689</v>
+      </c>
+      <c r="E56" t="s">
+        <v>690</v>
+      </c>
+      <c r="F56" t="s">
+        <v>633</v>
+      </c>
+      <c r="G56" t="s">
+        <v>691</v>
+      </c>
+      <c r="H56" t="s">
+        <v>692</v>
+      </c>
+      <c r="I56" t="s">
+        <v>692</v>
+      </c>
+      <c r="J56" t="s">
+        <v>693</v>
+      </c>
+      <c r="K56" t="s">
+        <v>684</v>
+      </c>
+      <c r="L56" t="s">
+        <v>684</v>
+      </c>
+      <c r="M56" t="s">
+        <v>53</v>
+      </c>
+      <c r="N56" t="s">
+        <v>54</v>
+      </c>
+      <c r="O56" t="s">
+        <v>55</v>
+      </c>
+      <c r="P56" t="s">
+        <v>318</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>179</v>
+      </c>
+      <c r="R56" t="s">
+        <v>479</v>
+      </c>
+      <c r="S56" t="s">
+        <v>49</v>
+      </c>
+      <c r="T56" t="s">
+        <v>480</v>
+      </c>
+      <c r="U56" t="s">
+        <v>57</v>
+      </c>
+      <c r="V56" t="s">
+        <v>57</v>
+      </c>
+      <c r="W56" t="s">
+        <v>164</v>
+      </c>
+      <c r="X56" t="s">
+        <v>481</v>
+      </c>
+      <c r="Y56" t="s">
+        <v>684</v>
+      </c>
+      <c r="Z56" t="s">
+        <v>482</v>
+      </c>
+      <c r="AA56" t="s">
+        <v>179</v>
+      </c>
+      <c r="AB56" t="s">
+        <v>694</v>
+      </c>
+      <c r="AC56" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD56" t="s">
+        <v>104</v>
+      </c>
+      <c r="AE56" t="s">
+        <v>84</v>
+      </c>
+      <c r="AF56" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG56" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH56" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI56" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ56" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK56" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL56" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM56" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN56" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO56" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP56" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="57" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>42</v>
+      </c>
+      <c r="B57" t="s">
+        <v>43</v>
+      </c>
+      <c r="C57" t="s">
+        <v>329</v>
+      </c>
+      <c r="D57" t="s">
+        <v>330</v>
+      </c>
+      <c r="E57" t="s">
+        <v>331</v>
+      </c>
+      <c r="F57" t="s">
+        <v>332</v>
+      </c>
+      <c r="G57" t="s">
+        <v>333</v>
+      </c>
+      <c r="H57" t="s">
+        <v>49</v>
+      </c>
+      <c r="I57" t="s">
+        <v>334</v>
+      </c>
+      <c r="J57" t="s">
+        <v>335</v>
+      </c>
+      <c r="K57" t="s">
+        <v>226</v>
+      </c>
+      <c r="L57" t="s">
+        <v>684</v>
+      </c>
+      <c r="M57" t="s">
+        <v>53</v>
+      </c>
+      <c r="N57" t="s">
+        <v>54</v>
+      </c>
+      <c r="O57" t="s">
+        <v>337</v>
+      </c>
+      <c r="P57" t="s">
+        <v>338</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>212</v>
+      </c>
+      <c r="R57" t="s">
+        <v>240</v>
+      </c>
+      <c r="S57" t="s">
+        <v>49</v>
+      </c>
+      <c r="T57" t="s">
+        <v>241</v>
+      </c>
+      <c r="U57" t="s">
+        <v>57</v>
+      </c>
+      <c r="V57" t="s">
+        <v>57</v>
+      </c>
+      <c r="W57" t="s">
+        <v>164</v>
+      </c>
+      <c r="X57" t="s">
+        <v>697</v>
+      </c>
+      <c r="Y57" t="s">
+        <v>684</v>
+      </c>
+      <c r="Z57" t="s">
+        <v>698</v>
+      </c>
+      <c r="AA57" t="s">
+        <v>259</v>
+      </c>
+      <c r="AB57" t="s">
+        <v>699</v>
+      </c>
+      <c r="AC57" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD57" t="s">
+        <v>126</v>
+      </c>
+      <c r="AE57" t="s">
+        <v>127</v>
+      </c>
+      <c r="AF57" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG57" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH57" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI57" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ57" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK57" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL57" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM57" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN57" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO57" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP57" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="58" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>42</v>
+      </c>
+      <c r="B58" t="s">
+        <v>43</v>
+      </c>
+      <c r="C58" t="s">
+        <v>701</v>
+      </c>
+      <c r="D58" t="s">
+        <v>702</v>
+      </c>
+      <c r="E58" t="s">
+        <v>703</v>
+      </c>
+      <c r="F58" t="s">
+        <v>173</v>
+      </c>
+      <c r="G58" t="s">
+        <v>704</v>
+      </c>
+      <c r="H58" t="s">
+        <v>705</v>
+      </c>
+      <c r="I58" t="s">
+        <v>705</v>
+      </c>
+      <c r="J58" t="s">
+        <v>706</v>
+      </c>
+      <c r="K58" t="s">
+        <v>684</v>
+      </c>
+      <c r="L58" t="s">
+        <v>684</v>
+      </c>
+      <c r="M58" t="s">
+        <v>53</v>
+      </c>
+      <c r="N58" t="s">
+        <v>54</v>
+      </c>
+      <c r="O58" t="s">
+        <v>55</v>
+      </c>
+      <c r="P58" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>57</v>
+      </c>
+      <c r="R58" t="s">
+        <v>707</v>
+      </c>
+      <c r="S58" t="s">
+        <v>49</v>
+      </c>
+      <c r="T58" t="s">
+        <v>708</v>
+      </c>
+      <c r="U58" t="s">
+        <v>57</v>
+      </c>
+      <c r="V58" t="s">
+        <v>57</v>
+      </c>
+      <c r="W58" t="s">
+        <v>60</v>
+      </c>
+      <c r="X58" t="s">
+        <v>707</v>
+      </c>
+      <c r="Y58" t="s">
+        <v>684</v>
+      </c>
+      <c r="Z58" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA58" t="s">
+        <v>381</v>
+      </c>
+      <c r="AB58" t="s">
+        <v>707</v>
+      </c>
+      <c r="AC58" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD58" t="s">
+        <v>229</v>
+      </c>
+      <c r="AE58" t="s">
+        <v>112</v>
+      </c>
+      <c r="AF58" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG58" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH58" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI58" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ58" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK58" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL58" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM58" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN58" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO58" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP58" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="59" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>42</v>
+      </c>
+      <c r="B59" t="s">
+        <v>43</v>
+      </c>
+      <c r="C59" t="s">
+        <v>710</v>
+      </c>
+      <c r="D59" t="s">
+        <v>711</v>
+      </c>
+      <c r="E59" t="s">
+        <v>712</v>
+      </c>
+      <c r="F59" t="s">
+        <v>173</v>
+      </c>
+      <c r="G59" t="s">
+        <v>704</v>
+      </c>
+      <c r="H59" t="s">
+        <v>49</v>
+      </c>
+      <c r="I59" t="s">
+        <v>713</v>
+      </c>
+      <c r="J59" t="s">
+        <v>714</v>
+      </c>
+      <c r="K59" t="s">
+        <v>684</v>
+      </c>
+      <c r="L59" t="s">
+        <v>715</v>
+      </c>
+      <c r="M59" t="s">
+        <v>53</v>
+      </c>
+      <c r="N59" t="s">
+        <v>54</v>
+      </c>
+      <c r="O59" t="s">
+        <v>55</v>
+      </c>
+      <c r="P59" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>57</v>
+      </c>
+      <c r="R59" t="s">
+        <v>707</v>
+      </c>
+      <c r="S59" t="s">
+        <v>49</v>
+      </c>
+      <c r="T59" t="s">
+        <v>708</v>
+      </c>
+      <c r="U59" t="s">
+        <v>57</v>
+      </c>
+      <c r="V59" t="s">
+        <v>57</v>
+      </c>
+      <c r="W59" t="s">
+        <v>60</v>
+      </c>
+      <c r="X59" t="s">
+        <v>707</v>
+      </c>
+      <c r="Y59" t="s">
+        <v>715</v>
+      </c>
+      <c r="Z59" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA59" t="s">
+        <v>239</v>
+      </c>
+      <c r="AB59" t="s">
+        <v>707</v>
+      </c>
+      <c r="AC59" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD59" t="s">
+        <v>229</v>
+      </c>
+      <c r="AE59" t="s">
+        <v>112</v>
+      </c>
+      <c r="AF59" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG59" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH59" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI59" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ59" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK59" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL59" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM59" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN59" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO59" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP59" t="s">
+        <v>716</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Actualizar CV_PF.xlsx — 26-03-2026, 11:53:47 a. m.
</commit_message>
<xml_diff>
--- a/datos/CV_PF.xlsx
+++ b/datos/CV_PF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{209904C7-2047-4A83-A536-14BE0857E281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC119C9A-4E9A-4ABA-81A6-6C4D1B44A38A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2730" uniqueCount="776">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2856" uniqueCount="810">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -2224,6 +2224,42 @@
     <t>3991</t>
   </si>
   <si>
+    <t>6839198-9</t>
+  </si>
+  <si>
+    <t>HERMOSILLA NORAMBUENA GRACIELA DEL CARMEN</t>
+  </si>
+  <si>
+    <t>05/01/1949</t>
+  </si>
+  <si>
+    <t>La Pintana</t>
+  </si>
+  <si>
+    <t>11122 - La Pintana - Santiago -CP</t>
+  </si>
+  <si>
+    <t>987418795</t>
+  </si>
+  <si>
+    <t>mana2010@live.cl; ; ; ;</t>
+  </si>
+  <si>
+    <t>Nayaret tatiana puga marchant</t>
+  </si>
+  <si>
+    <t>1344538</t>
+  </si>
+  <si>
+    <t>500000</t>
+  </si>
+  <si>
+    <t>18644</t>
+  </si>
+  <si>
+    <t>3992</t>
+  </si>
+  <si>
     <t>11399404-5</t>
   </si>
   <si>
@@ -2242,9 +2278,6 @@
     <t>edelmiraguerraleiv@gmail.com; ; ; ;</t>
   </si>
   <si>
-    <t>Nayaret tatiana puga marchant</t>
-  </si>
-  <si>
     <t>0.08</t>
   </si>
   <si>
@@ -2348,6 +2381,75 @@
   </si>
   <si>
     <t>3999</t>
+  </si>
+  <si>
+    <t>14715130-6</t>
+  </si>
+  <si>
+    <t>VALAREZO MACIAS LAURA  ANGELINA</t>
+  </si>
+  <si>
+    <t>25/03/1976</t>
+  </si>
+  <si>
+    <t>Santo Domingo</t>
+  </si>
+  <si>
+    <t>101 - Santo Domingo - San Antonio -CP</t>
+  </si>
+  <si>
+    <t>992376457</t>
+  </si>
+  <si>
+    <t>laura_valarezo@yahoo.es; ; ; ;</t>
+  </si>
+  <si>
+    <t>25/03/2026</t>
+  </si>
+  <si>
+    <t>6630000</t>
+  </si>
+  <si>
+    <t>5571429</t>
+  </si>
+  <si>
+    <t>663000</t>
+  </si>
+  <si>
+    <t>5967000</t>
+  </si>
+  <si>
+    <t>165750</t>
+  </si>
+  <si>
+    <t>SERVICIO FUNERARIO TESOROS DEL ALMA SOLUCIÓN TOTAL FAMILIAR</t>
+  </si>
+  <si>
+    <t>4002</t>
+  </si>
+  <si>
+    <t>22010293-9</t>
+  </si>
+  <si>
+    <t>AVILA CANDIA CAMILA VALERIA</t>
+  </si>
+  <si>
+    <t>29/12/2005</t>
+  </si>
+  <si>
+    <t>239 - San Bernardo - Maipo -CP</t>
+  </si>
+  <si>
+    <t>990934743</t>
+  </si>
+  <si>
+    <t>camila.avila.candia@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>4003</t>
   </si>
 </sst>
 </file>
@@ -3208,10 +3310,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP65"/>
+  <dimension ref="A1:AP68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="42" width="8" customWidth="1"/>
+    <col min="1" max="41" width="8" customWidth="1"/>
+    <col min="42" max="42" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.3">
@@ -8548,7 +8651,7 @@
         <v>555</v>
       </c>
       <c r="AC42" t="s">
-        <v>103</v>
+        <v>62</v>
       </c>
       <c r="AD42" t="s">
         <v>311</v>
@@ -9649,7 +9752,7 @@
         <v>423</v>
       </c>
       <c r="L51" t="s">
-        <v>479</v>
+        <v>568</v>
       </c>
       <c r="M51" t="s">
         <v>53</v>
@@ -10084,7 +10187,7 @@
         <v>687</v>
       </c>
       <c r="AC54" t="s">
-        <v>103</v>
+        <v>62</v>
       </c>
       <c r="AD54" t="s">
         <v>104</v>
@@ -11039,25 +11142,25 @@
         <v>736</v>
       </c>
       <c r="F62" t="s">
-        <v>157</v>
+        <v>737</v>
       </c>
       <c r="G62" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="H62" t="s">
         <v>49</v>
       </c>
       <c r="I62" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="J62" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="K62" t="s">
-        <v>717</v>
+        <v>660</v>
       </c>
       <c r="L62" t="s">
-        <v>717</v>
+        <v>660</v>
       </c>
       <c r="M62" t="s">
         <v>53</v>
@@ -11069,19 +11172,19 @@
         <v>399</v>
       </c>
       <c r="P62" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="Q62" t="s">
         <v>627</v>
       </c>
       <c r="R62" t="s">
-        <v>483</v>
+        <v>513</v>
       </c>
       <c r="S62" t="s">
         <v>49</v>
       </c>
       <c r="T62" t="s">
-        <v>512</v>
+        <v>742</v>
       </c>
       <c r="U62" t="s">
         <v>57</v>
@@ -11090,19 +11193,19 @@
         <v>57</v>
       </c>
       <c r="W62" t="s">
-        <v>741</v>
+        <v>182</v>
       </c>
       <c r="X62" t="s">
-        <v>165</v>
+        <v>743</v>
       </c>
       <c r="Y62" t="s">
-        <v>717</v>
+        <v>660</v>
       </c>
       <c r="Z62" t="s">
-        <v>742</v>
+        <v>469</v>
       </c>
       <c r="AA62" t="s">
-        <v>743</v>
+        <v>309</v>
       </c>
       <c r="AB62" t="s">
         <v>744</v>
@@ -11111,10 +11214,10 @@
         <v>103</v>
       </c>
       <c r="AD62" t="s">
-        <v>111</v>
+        <v>516</v>
       </c>
       <c r="AE62" t="s">
-        <v>112</v>
+        <v>312</v>
       </c>
       <c r="AF62" t="s">
         <v>65</v>
@@ -11167,22 +11270,22 @@
         <v>748</v>
       </c>
       <c r="F63" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="G63" t="s">
-        <v>705</v>
+        <v>749</v>
       </c>
       <c r="H63" t="s">
         <v>49</v>
       </c>
       <c r="I63" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="J63" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="K63" t="s">
-        <v>685</v>
+        <v>717</v>
       </c>
       <c r="L63" t="s">
         <v>717</v>
@@ -11194,22 +11297,22 @@
         <v>54</v>
       </c>
       <c r="O63" t="s">
-        <v>55</v>
+        <v>399</v>
       </c>
       <c r="P63" t="s">
-        <v>94</v>
+        <v>741</v>
       </c>
       <c r="Q63" t="s">
-        <v>57</v>
+        <v>627</v>
       </c>
       <c r="R63" t="s">
-        <v>708</v>
+        <v>483</v>
       </c>
       <c r="S63" t="s">
         <v>49</v>
       </c>
       <c r="T63" t="s">
-        <v>709</v>
+        <v>512</v>
       </c>
       <c r="U63" t="s">
         <v>57</v>
@@ -11218,28 +11321,28 @@
         <v>57</v>
       </c>
       <c r="W63" t="s">
-        <v>60</v>
+        <v>752</v>
       </c>
       <c r="X63" t="s">
-        <v>708</v>
+        <v>165</v>
       </c>
       <c r="Y63" t="s">
         <v>717</v>
       </c>
       <c r="Z63" t="s">
-        <v>49</v>
+        <v>753</v>
       </c>
       <c r="AA63" t="s">
-        <v>241</v>
+        <v>754</v>
       </c>
       <c r="AB63" t="s">
-        <v>708</v>
+        <v>755</v>
       </c>
       <c r="AC63" t="s">
-        <v>62</v>
+        <v>103</v>
       </c>
       <c r="AD63" t="s">
-        <v>231</v>
+        <v>111</v>
       </c>
       <c r="AE63" t="s">
         <v>112</v>
@@ -11275,7 +11378,7 @@
         <v>49</v>
       </c>
       <c r="AP63" t="s">
-        <v>751</v>
+        <v>756</v>
       </c>
     </row>
     <row r="64" spans="1:42" x14ac:dyDescent="0.3">
@@ -11286,34 +11389,34 @@
         <v>43</v>
       </c>
       <c r="C64" t="s">
-        <v>752</v>
+        <v>757</v>
       </c>
       <c r="D64" t="s">
-        <v>753</v>
+        <v>758</v>
       </c>
       <c r="E64" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="F64" t="s">
-        <v>269</v>
+        <v>173</v>
       </c>
       <c r="G64" t="s">
-        <v>755</v>
+        <v>705</v>
       </c>
       <c r="H64" t="s">
         <v>49</v>
       </c>
       <c r="I64" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="J64" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="K64" t="s">
-        <v>625</v>
+        <v>685</v>
       </c>
       <c r="L64" t="s">
-        <v>625</v>
+        <v>717</v>
       </c>
       <c r="M64" t="s">
         <v>53</v>
@@ -11322,22 +11425,22 @@
         <v>54</v>
       </c>
       <c r="O64" t="s">
-        <v>140</v>
+        <v>55</v>
       </c>
       <c r="P64" t="s">
-        <v>758</v>
+        <v>94</v>
       </c>
       <c r="Q64" t="s">
-        <v>212</v>
+        <v>57</v>
       </c>
       <c r="R64" t="s">
-        <v>759</v>
+        <v>708</v>
       </c>
       <c r="S64" t="s">
         <v>49</v>
       </c>
       <c r="T64" t="s">
-        <v>760</v>
+        <v>709</v>
       </c>
       <c r="U64" t="s">
         <v>57</v>
@@ -11346,25 +11449,25 @@
         <v>57</v>
       </c>
       <c r="W64" t="s">
-        <v>164</v>
+        <v>60</v>
       </c>
       <c r="X64" t="s">
-        <v>761</v>
+        <v>708</v>
       </c>
       <c r="Y64" t="s">
-        <v>625</v>
+        <v>717</v>
       </c>
       <c r="Z64" t="s">
-        <v>762</v>
+        <v>49</v>
       </c>
       <c r="AA64" t="s">
-        <v>343</v>
+        <v>241</v>
       </c>
       <c r="AB64" t="s">
-        <v>763</v>
+        <v>708</v>
       </c>
       <c r="AC64" t="s">
-        <v>103</v>
+        <v>62</v>
       </c>
       <c r="AD64" t="s">
         <v>231</v>
@@ -11403,7 +11506,7 @@
         <v>49</v>
       </c>
       <c r="AP64" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
     </row>
     <row r="65" spans="1:42" x14ac:dyDescent="0.3">
@@ -11414,34 +11517,34 @@
         <v>43</v>
       </c>
       <c r="C65" t="s">
+        <v>763</v>
+      </c>
+      <c r="D65" t="s">
+        <v>764</v>
+      </c>
+      <c r="E65" t="s">
         <v>765</v>
       </c>
-      <c r="D65" t="s">
+      <c r="F65" t="s">
+        <v>269</v>
+      </c>
+      <c r="G65" t="s">
         <v>766</v>
       </c>
-      <c r="E65" t="s">
+      <c r="H65" t="s">
+        <v>49</v>
+      </c>
+      <c r="I65" t="s">
         <v>767</v>
       </c>
-      <c r="F65" t="s">
+      <c r="J65" t="s">
         <v>768</v>
       </c>
-      <c r="G65" t="s">
-        <v>769</v>
-      </c>
-      <c r="H65" t="s">
-        <v>770</v>
-      </c>
-      <c r="I65" t="s">
-        <v>770</v>
-      </c>
-      <c r="J65" t="s">
-        <v>771</v>
-      </c>
       <c r="K65" t="s">
-        <v>568</v>
+        <v>625</v>
       </c>
       <c r="L65" t="s">
-        <v>568</v>
+        <v>625</v>
       </c>
       <c r="M65" t="s">
         <v>53</v>
@@ -11453,19 +11556,19 @@
         <v>140</v>
       </c>
       <c r="P65" t="s">
-        <v>240</v>
+        <v>769</v>
       </c>
       <c r="Q65" t="s">
-        <v>143</v>
+        <v>212</v>
       </c>
       <c r="R65" t="s">
-        <v>593</v>
+        <v>770</v>
       </c>
       <c r="S65" t="s">
         <v>49</v>
       </c>
       <c r="T65" t="s">
-        <v>594</v>
+        <v>771</v>
       </c>
       <c r="U65" t="s">
         <v>57</v>
@@ -11480,7 +11583,7 @@
         <v>772</v>
       </c>
       <c r="Y65" t="s">
-        <v>568</v>
+        <v>625</v>
       </c>
       <c r="Z65" t="s">
         <v>773</v>
@@ -11495,10 +11598,10 @@
         <v>103</v>
       </c>
       <c r="AD65" t="s">
-        <v>328</v>
+        <v>231</v>
       </c>
       <c r="AE65" t="s">
-        <v>329</v>
+        <v>112</v>
       </c>
       <c r="AF65" t="s">
         <v>65</v>
@@ -11532,6 +11635,390 @@
       </c>
       <c r="AP65" t="s">
         <v>775</v>
+      </c>
+    </row>
+    <row r="66" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>42</v>
+      </c>
+      <c r="B66" t="s">
+        <v>43</v>
+      </c>
+      <c r="C66" t="s">
+        <v>776</v>
+      </c>
+      <c r="D66" t="s">
+        <v>777</v>
+      </c>
+      <c r="E66" t="s">
+        <v>778</v>
+      </c>
+      <c r="F66" t="s">
+        <v>779</v>
+      </c>
+      <c r="G66" t="s">
+        <v>780</v>
+      </c>
+      <c r="H66" t="s">
+        <v>781</v>
+      </c>
+      <c r="I66" t="s">
+        <v>781</v>
+      </c>
+      <c r="J66" t="s">
+        <v>782</v>
+      </c>
+      <c r="K66" t="s">
+        <v>568</v>
+      </c>
+      <c r="L66" t="s">
+        <v>568</v>
+      </c>
+      <c r="M66" t="s">
+        <v>53</v>
+      </c>
+      <c r="N66" t="s">
+        <v>54</v>
+      </c>
+      <c r="O66" t="s">
+        <v>140</v>
+      </c>
+      <c r="P66" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q66" t="s">
+        <v>143</v>
+      </c>
+      <c r="R66" t="s">
+        <v>593</v>
+      </c>
+      <c r="S66" t="s">
+        <v>49</v>
+      </c>
+      <c r="T66" t="s">
+        <v>594</v>
+      </c>
+      <c r="U66" t="s">
+        <v>57</v>
+      </c>
+      <c r="V66" t="s">
+        <v>57</v>
+      </c>
+      <c r="W66" t="s">
+        <v>164</v>
+      </c>
+      <c r="X66" t="s">
+        <v>783</v>
+      </c>
+      <c r="Y66" t="s">
+        <v>568</v>
+      </c>
+      <c r="Z66" t="s">
+        <v>784</v>
+      </c>
+      <c r="AA66" t="s">
+        <v>343</v>
+      </c>
+      <c r="AB66" t="s">
+        <v>785</v>
+      </c>
+      <c r="AC66" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD66" t="s">
+        <v>328</v>
+      </c>
+      <c r="AE66" t="s">
+        <v>329</v>
+      </c>
+      <c r="AF66" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG66" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH66" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI66" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ66" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK66" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL66" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM66" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN66" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO66" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP66" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="67" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>42</v>
+      </c>
+      <c r="B67" t="s">
+        <v>501</v>
+      </c>
+      <c r="C67" t="s">
+        <v>787</v>
+      </c>
+      <c r="D67" t="s">
+        <v>788</v>
+      </c>
+      <c r="E67" t="s">
+        <v>789</v>
+      </c>
+      <c r="F67" t="s">
+        <v>790</v>
+      </c>
+      <c r="G67" t="s">
+        <v>791</v>
+      </c>
+      <c r="H67" t="s">
+        <v>49</v>
+      </c>
+      <c r="I67" t="s">
+        <v>792</v>
+      </c>
+      <c r="J67" t="s">
+        <v>793</v>
+      </c>
+      <c r="K67" t="s">
+        <v>479</v>
+      </c>
+      <c r="L67" t="s">
+        <v>794</v>
+      </c>
+      <c r="M67" t="s">
+        <v>53</v>
+      </c>
+      <c r="N67" t="s">
+        <v>54</v>
+      </c>
+      <c r="O67" t="s">
+        <v>339</v>
+      </c>
+      <c r="P67" t="s">
+        <v>340</v>
+      </c>
+      <c r="Q67" t="s">
+        <v>212</v>
+      </c>
+      <c r="R67" t="s">
+        <v>795</v>
+      </c>
+      <c r="S67" t="s">
+        <v>49</v>
+      </c>
+      <c r="T67" t="s">
+        <v>796</v>
+      </c>
+      <c r="U67" t="s">
+        <v>57</v>
+      </c>
+      <c r="V67" t="s">
+        <v>57</v>
+      </c>
+      <c r="W67" t="s">
+        <v>164</v>
+      </c>
+      <c r="X67" t="s">
+        <v>797</v>
+      </c>
+      <c r="Y67" t="s">
+        <v>794</v>
+      </c>
+      <c r="Z67" t="s">
+        <v>798</v>
+      </c>
+      <c r="AA67" t="s">
+        <v>651</v>
+      </c>
+      <c r="AB67" t="s">
+        <v>799</v>
+      </c>
+      <c r="AC67" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD67" t="s">
+        <v>800</v>
+      </c>
+      <c r="AE67" t="s">
+        <v>457</v>
+      </c>
+      <c r="AF67" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG67" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH67" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI67" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ67" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK67" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL67" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM67" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN67" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO67" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP67" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="68" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>42</v>
+      </c>
+      <c r="B68" t="s">
+        <v>43</v>
+      </c>
+      <c r="C68" t="s">
+        <v>802</v>
+      </c>
+      <c r="D68" t="s">
+        <v>803</v>
+      </c>
+      <c r="E68" t="s">
+        <v>804</v>
+      </c>
+      <c r="F68" t="s">
+        <v>372</v>
+      </c>
+      <c r="G68" t="s">
+        <v>805</v>
+      </c>
+      <c r="H68" t="s">
+        <v>49</v>
+      </c>
+      <c r="I68" t="s">
+        <v>806</v>
+      </c>
+      <c r="J68" t="s">
+        <v>807</v>
+      </c>
+      <c r="K68" t="s">
+        <v>613</v>
+      </c>
+      <c r="L68" t="s">
+        <v>613</v>
+      </c>
+      <c r="M68" t="s">
+        <v>53</v>
+      </c>
+      <c r="N68" t="s">
+        <v>54</v>
+      </c>
+      <c r="O68" t="s">
+        <v>55</v>
+      </c>
+      <c r="P68" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>57</v>
+      </c>
+      <c r="R68" t="s">
+        <v>469</v>
+      </c>
+      <c r="S68" t="s">
+        <v>49</v>
+      </c>
+      <c r="T68" t="s">
+        <v>569</v>
+      </c>
+      <c r="U68" t="s">
+        <v>57</v>
+      </c>
+      <c r="V68" t="s">
+        <v>57</v>
+      </c>
+      <c r="W68" t="s">
+        <v>60</v>
+      </c>
+      <c r="X68" t="s">
+        <v>469</v>
+      </c>
+      <c r="Y68" t="s">
+        <v>613</v>
+      </c>
+      <c r="Z68" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA68" t="s">
+        <v>808</v>
+      </c>
+      <c r="AB68" t="s">
+        <v>469</v>
+      </c>
+      <c r="AC68" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD68" t="s">
+        <v>231</v>
+      </c>
+      <c r="AE68" t="s">
+        <v>112</v>
+      </c>
+      <c r="AF68" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG68" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH68" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI68" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ68" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK68" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL68" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM68" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN68" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO68" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP68" t="s">
+        <v>809</v>
       </c>
     </row>
   </sheetData>

</xml_diff>